<commit_message>
Add paper 680014 to session 44
AI-Powered Intraday Trading System Using Diffusion-Based Time-Series Modeling (Camera
Ready Done) is scheduled for Tuesday at the committee's request. Every Tuesday
10:00 session is full, and a seventh paper there would run into the 11:12 break. It
is appended to session 44, Representation Learning, Generative and Numerical Methods,
which suits diffusion-based modelling, at 12:37. The session now ends at 12:49, three
minutes before the Valedictory, as sessions 22 and 60 already do. No other paper
moves. verify-17.js expects 383 papers and passes. The session 44 chair sheet is
regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/programme/chair-sheets/S44.xlsx
+++ b/programme/chair-sheets/S44.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t xml:space="preserve">ICCCMLA 2026 - Session attendance and evaluation sheet</t>
   </si>
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Date and time</t>
   </si>
   <si>
-    <t xml:space="preserve">Tuesday, 6 October 2026, 11:25-12:37 IST (Room K)</t>
+    <t xml:space="preserve">Tuesday, 6 October 2026, 11:25-12:49 IST (Room K)</t>
   </si>
   <si>
     <t xml:space="preserve">Session chair</t>
@@ -149,6 +149,15 @@
   </si>
   <si>
     <t xml:space="preserve">DYNAMIC REWARD TOPOLOGY: SELF-SUPERVISED TRAJECTORY GENERATION FOR SPARSE-REWARD MULTI-AGENT REINFORCEMENT LEARNING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:37-12:49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">680014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI-Powered Intraday Trading System Using Diffusion-Based Time-Series Modeling</t>
   </si>
   <si>
     <t xml:space="preserve">Papers scheduled</t>
@@ -663,7 +672,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -966,81 +975,94 @@
       <c r="K16" s="9"/>
       <c r="L16" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="3" t="s">
+    <row r="17" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="12" t="n">
-        <f aca="false">COUNTA(C11:C16)</f>
-        <v>6</v>
-      </c>
+      <c r="C17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="11" t="str">
+        <f aca="false">IF(COUNT(G17:I17)=0,"",SUM(G17:I17))</f>
+        <v/>
+      </c>
+      <c r="K17" s="9"/>
+      <c r="L17" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="12" t="n">
-        <f aca="false">COUNTIF(E11:E16,"Present")</f>
-        <v>0</v>
+        <f aca="false">COUNTA(C11:C17)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="12" t="n">
-        <f aca="false">COUNTIF(E11:E16,"Late")</f>
+        <f aca="false">COUNTIF(E11:E17,"Present")</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C21" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="12" t="n">
-        <f aca="false">COUNTIF(E11:E16,"Absent")</f>
+        <f aca="false">COUNTIF(E11:E17,"Late")</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C22" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="12" t="n">
-        <f aca="false">COUNTA(C11:C16)-COUNTA(E11:E16)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF(E11:E17,"Absent")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="12" t="n">
-        <f aca="false">COUNTIF(K11:K16,"Yes")</f>
+        <f aca="false">COUNTA(C11:C17)-COUNTA(E11:E17)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C24" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="3"/>
+      <c r="E24" s="12" t="n">
+        <f aca="false">COUNTIF(K11:K17,"Yes")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1052,7 +1074,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1064,7 +1086,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1074,9 +1096,9 @@
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
     </row>
-    <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1086,25 +1108,21 @@
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
     </row>
-    <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
+    <row r="30" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -1120,7 +1138,7 @@
     </row>
     <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -1136,7 +1154,7 @@
     </row>
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -1152,7 +1170,7 @@
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -1165,6 +1183,22 @@
       <c r="J35" s="14"/>
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
+    </row>
+    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="14"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
+      <c r="L36" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -1178,14 +1212,12 @@
     <mergeCell ref="C7:L7"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:L8"/>
-    <mergeCell ref="C18:D18"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="C23:D23"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="D25:H25"/>
+    <mergeCell ref="C24:D24"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="D26:H26"/>
     <mergeCell ref="A27:C27"/>
@@ -1194,22 +1226,24 @@
     <mergeCell ref="D28:H28"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="D29:H29"/>
-    <mergeCell ref="A31:L31"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="D30:H30"/>
     <mergeCell ref="A32:L32"/>
     <mergeCell ref="A33:L33"/>
     <mergeCell ref="A34:L34"/>
     <mergeCell ref="A35:L35"/>
+    <mergeCell ref="A36:L36"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E11:E16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E11:E17" type="list">
       <formula1>"Present,Late,Absent"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a whole number from 0 to 10." errorStyle="stop" errorTitle="Score" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G11:I16" type="whole">
+    <dataValidation allowBlank="true" error="Enter a whole number from 0 to 10." errorStyle="stop" errorTitle="Score" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G11:I17" type="whole">
       <formula1>0</formula1>
       <formula2>10</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K16" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K11:K17" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>